<commit_message>
feat: add SetSubtotal API for pivot field subtotal management
Add IXLPivotField.SetSubtotal(XLSubtotalFunction, bool) to enable
adding and removing individual subtotal functions. Changes subtotal
semantics: empty collection = no subtotals, Automatic = default
subtotal. Previously empty meant default, which made it impossible
to remove subtotals from a field.

Inspired by ClosedXML/ClosedXML#1821

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PivotTables/PivotTables.xlsx
+++ b/XLibur.Tests/Resource/Examples/PivotTables/PivotTables.xlsx
@@ -149,27 +149,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvt" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisCol" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField name="Month" axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="0"/>
@@ -193,37 +195,40 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtInteger" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="5">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField name="Code" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="6">
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Code" axis="axisRow" showAll="0">
+      <items count="7">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField name="BakeDate" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="16">
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="BakeDate" axis="axisRow" showAll="0">
+      <items count="17">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -240,6 +245,7 @@
         <item x="13"/>
         <item x="14"/>
         <item x="15"/>
+        <item t="default"/>
       </items>
     </pivotField>
   </pivotFields>
@@ -269,27 +275,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvt" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisCol" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="-2"/>
@@ -315,27 +323,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvt" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisCol" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="0"/>
@@ -362,27 +372,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtNoColumnLabels" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1" rowHeaderCaption="Pastry name">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="0"/>
@@ -408,27 +420,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtCollapsedFields" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0">
+      <items count="6">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisRow" showAll="0">
       <items count="5">
         <item sd="0" x="0"/>
         <item sd="0" x="1"/>
         <item sd="0" x="2"/>
         <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default" sd="0"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="0"/>
@@ -454,27 +468,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtFieldAsValueAndLabel" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" dataField="1" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" dataField="1" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField name="Month" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="0"/>
@@ -496,27 +512,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtHidesubTotals" cacheId="0" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1" colHeaderCaption="Measures">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisCol" showAll="0" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisCol" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisCol" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisCol" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="-2"/>
@@ -542,20 +560,19 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtFilter" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1">
   <location ref="A5" firstHeaderRow="0" firstDataRow="0" firstDataCol="0" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="6">
+    <pivotField name="Name" axis="axisPage" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
+      <items count="5">
         <item h="1" x="0"/>
         <item x="1"/>
         <item h="1" x="2"/>
         <item h="1" x="3"/>
         <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Quality" axis="axisPage" showAll="0">
-      <items count="17">
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Quality" axis="axisPage" showAll="0" defaultSubtotal="0">
+      <items count="16">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -572,19 +589,19 @@
         <item x="13"/>
         <item x="14"/>
         <item x="15"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name="Month" axis="axisRow" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField name="BakeDate" axis="axisPage" showAll="0">
-      <items count="17">
+      </items>
+    </pivotField>
+    <pivotField name="Month" axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="BakeDate" axis="axisPage" showAll="0" defaultSubtotal="0">
+      <items count="16">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -601,7 +618,6 @@
         <item x="13"/>
         <item x="14"/>
         <item x="15"/>
-        <item t="default"/>
       </items>
     </pivotField>
   </pivotFields>
@@ -629,27 +645,29 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="pvtSort" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" outline="1" rowHeaderCaption="Pastry name">
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="6">
-    <pivotField name="Name" axis="axisRow" showAll="0" sortType="ascending" defaultSubtotal="0">
+    <pivotField name="Name" axis="axisRow" showAll="0" sortType="ascending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
+    <pivotField name="Month" axis="axisRow" showAll="0" sortType="descending">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField name="Month" axis="axisRow" showAll="0" sortType="descending" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="0"/>

</xml_diff>